<commit_message>
Add new exercises for string manipulation, digit counting, and basic calculations
</commit_message>
<xml_diff>
--- a/docs/python/LOGIC_BUILDING_PYTHON.xlsx
+++ b/docs/python/LOGIC_BUILDING_PYTHON.xlsx
@@ -3405,7 +3405,7 @@
       </c>
       <c r="C133" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18">
       <c r="A134" s="12" t="s">
         <v>218</v>
       </c>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="C134" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18">
       <c r="A135" s="9" t="s">
         <v>219</v>
       </c>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="C135" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18">
       <c r="A136" s="12" t="s">
         <v>220</v>
       </c>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="C136" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18">
       <c r="A137" s="9" t="s">
         <v>221</v>
       </c>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="C137" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18">
       <c r="A138" s="12" t="s">
         <v>222</v>
       </c>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="C138" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18">
       <c r="A139" s="9" t="s">
         <v>223</v>
       </c>
@@ -3461,7 +3461,7 @@
         <v>123</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18">
       <c r="A140" s="12" t="s">
         <v>224</v>
       </c>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="C140" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18">
       <c r="A141" s="9" t="s">
         <v>225</v>
       </c>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="C141" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18">
       <c r="A142" s="12" t="s">
         <v>226</v>
       </c>
@@ -3488,7 +3488,7 @@
       </c>
       <c r="C142" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18">
       <c r="A143" s="9" t="s">
         <v>227</v>
       </c>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="C143" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18">
       <c r="A144" s="12" t="s">
         <v>228</v>
       </c>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="C144" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18">
       <c r="A145" s="9" t="s">
         <v>229</v>
       </c>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="C145" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18">
       <c r="A146" s="12" t="s">
         <v>230</v>
       </c>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="C146" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18">
       <c r="A147" s="9" t="s">
         <v>231</v>
       </c>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C147" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18">
       <c r="A148" s="12" t="s">
         <v>232</v>
       </c>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="C148" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18">
       <c r="A149" s="9" t="s">
         <v>233</v>
       </c>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="C149" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18">
       <c r="A150" s="12" t="s">
         <v>234</v>
       </c>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="C150" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18">
       <c r="A151" s="9" t="s">
         <v>235</v>
       </c>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="C151" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18">
       <c r="A152" s="12" t="s">
         <v>236</v>
       </c>

</xml_diff>

<commit_message>
Refactor logic building exercises in Python: - Added examples and improved comments for clarity in exercises 58 to 99. - Updated input prompts and output messages for better user experience. - Ensured consistent formatting and structure across all exercises. - Removed unnecessary comments and improved readability.
</commit_message>
<xml_diff>
--- a/docs/python/LOGIC_BUILDING_PYTHON.xlsx
+++ b/docs/python/LOGIC_BUILDING_PYTHON.xlsx
@@ -3578,7 +3578,7 @@
       </c>
       <c r="C152" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18">
       <c r="A153" s="9" t="s">
         <v>237</v>
       </c>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="C153" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18">
       <c r="A154" s="12" t="s">
         <v>238</v>
       </c>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="C154" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="32">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18">
       <c r="A155" s="9" t="s">
         <v>239</v>
       </c>

</xml_diff>